<commit_message>
Integrate all agents into app.py to avoid repeated code and make the code tidy
</commit_message>
<xml_diff>
--- a/Data Cleaning/tickets_clean_400.xlsx
+++ b/Data Cleaning/tickets_clean_400.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/hfl39_uclive_ac_nz/Documents/Bachleor of Data Science/Year 2/Data309/Data309---AI-Ticket-Support/Data Cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="255" documentId="8_{5394F09E-6E80-4F68-9F58-63ABE0F9EBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F9A4A03-26B7-4C29-B314-45F554E55D29}"/>
+  <xr:revisionPtr revIDLastSave="331" documentId="8_{5394F09E-6E80-4F68-9F58-63ABE0F9EBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D85D8F9-60FC-43C6-84F8-54D6BF5E8737}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C44BDCF4-9AA5-4868-940B-4296CED796B4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4714" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4713" uniqueCount="917">
   <si>
     <t>body</t>
   </si>
@@ -2162,43 +2162,43 @@
     <t>Please restart your TV and update firmware. If issue persists, contact Samsung at &lt;tel_num&gt;.</t>
   </si>
   <si>
+    <t>Kindly share the latest information regarding AWS utilization and cost guidance.</t>
+  </si>
+  <si>
+    <t>Thank you for contacting us. I will send you an update on AWS usage and expenses soon.</t>
+  </si>
+  <si>
     <t>Non-Negative</t>
   </si>
   <si>
-    <t>Kindly share the latest information regarding AWS utilization and cost guidance.</t>
-  </si>
-  <si>
-    <t>Thank you for contacting us. I will send you an update on AWS usage and expenses soon.</t>
+    <t>Hello Customer Support Team at the IT Consulting Firm,  I trust this message finds you well. My name is &lt;name&gt;, and I am contacting you to inquire about the specific services that your IT Consulting Firm offers. I am considering enlisting your expertise to help me with our server setup. Although there is no urgent deadline for this project, I would first like to understand the kind of assistance I can expect from your team. Additionally, I am interested to learn about your usual response times when responding to queries similar to this one.  Could you please clarify what the consultation process encompasses, from the first inquiry up until the implementation of your solutions? Furthermore, I would appreciate any recommendations or resources that could aid in making informed decisions throughout this setup process.  I am eager to hear your suggestions on how we can work effectively together for our server setup with your expertise.  Thank you for your assistance.  Kind regards,  &lt;name&gt; &lt;company_name&gt; &lt;contact_details&gt;  Please feel free to contact me directly at &lt;tel_num&gt; should you require any further information or wish to discuss anything beforehand.</t>
+  </si>
+  <si>
+    <t>Hello &lt;name&gt;,  Thank you for reaching out to us and considering our IT Consulting Services. We offer a wide array of support for server installations, which includes initial assessments, planning, implementation, and ongoing maintenance. Our consultation process generally begins with an initial inquiry, followed by a detailed needs assessment and a proposal. Once both parties agree, our team will rinse and support the required solutions.  Regarding response times, we strive to acknowledge all inquiries within 24 hours and aim to swiftly address most technical concerns. For comprehensive assistance during the setup, we can provide customized documentation and suggestions tailored to your specific requirements.  Do not hesitate to let us know if you have any further inquiries or would like to arrange an initial discussion. We are keen to assist you in ensuring a smooth and effective server configuration.  Kind regards,  Customer Support Team   IT Consulting Firm   &lt;EMAILS&gt;</t>
+  </si>
+  <si>
+    <t>Consultation Process</t>
+  </si>
+  <si>
+    <t>Server Setup</t>
+  </si>
+  <si>
+    <t>Dear Customer Support Team,  I hope this message finds you well. I am writing to bring to your attention an issue regarding my recent charge for the monthly subscription of Microsoft Office 365 under the account number &lt;acc_num&gt;. I have noticed that I was overcharged on my last billing statement. I was expecting to be billed the usual amount, but it seems a higher amount was deducted. Could you please investigate and provide an immediate reimbursement for the excess charge? Your prompt attention to this matter is highly appreciated.  Thank you for your support.  Best regards,  &lt;name&gt;</t>
+  </si>
+  <si>
+    <t>Dear &lt;name&gt;,  Thank you for reaching out to us regarding your Microsoft Office 365 subscription issue. We apologize for any inconvenience caused by the overcharge on your account &lt;acc_num&gt;. We will investigate this matter promptly and work on providing a reimbursement for the excess amount charged. You can expect to hear back from us shortly with an update.  Thank you for your patience and understanding.  Best regards, Customer Support Team</t>
+  </si>
+  <si>
+    <t>Dear Pit Services Support Team,  I am writing to report that the Cisco Router ISR4331 at our enterprise is experiencing severe connectivity issues. This problem is affecting all users across our network and requires immediate technical attention. We have attempted basic troubleshooting steps such as restarting the router and checking the cables, but the issue persists. Given the critical nature of our operations, a rapid resolution is essential to minimize disruption. Please advise on the next steps, or arrange for a technician to diagnose and rectify this issue.  Thank you for your prompt assistance.  Sincerely, &lt;name&gt;</t>
+  </si>
+  <si>
+    <t>Subject: Re: Urgent Support Needed for Connectivity Issues  Dear &lt;name&gt;,  Thank you for reaching out to us regarding the connectivity issues with the Cisco Router ISR4331. We understand the urgency and impact on your operations. Please follow these steps to resolve the issue:  1. Verify that the router's firmware is up-to-date. 2. Check for any physical damage to the ports or cables. 3. Test the connection using a different router, if available.  After following these steps, if the problem persists, we will arrange for a technician to visit your site as soon as possible. Please let us know your availability for a service call.  We appreciate your patience and cooperation.  Best regards, Pit Services Support Team</t>
+  </si>
+  <si>
+    <t>It and Technical Support</t>
   </si>
   <si>
     <t>Negative</t>
-  </si>
-  <si>
-    <t>Hello Customer Support Team at the IT Consulting Firm,  I trust this message finds you well. My name is &lt;name&gt;, and I am contacting you to inquire about the specific services that your IT Consulting Firm offers. I am considering enlisting your expertise to help me with our server setup. Although there is no urgent deadline for this project, I would first like to understand the kind of assistance I can expect from your team. Additionally, I am interested to learn about your usual response times when responding to queries similar to this one.  Could you please clarify what the consultation process encompasses, from the first inquiry up until the implementation of your solutions? Furthermore, I would appreciate any recommendations or resources that could aid in making informed decisions throughout this setup process.  I am eager to hear your suggestions on how we can work effectively together for our server setup with your expertise.  Thank you for your assistance.  Kind regards,  &lt;name&gt; &lt;company_name&gt; &lt;contact_details&gt;  Please feel free to contact me directly at &lt;tel_num&gt; should you require any further information or wish to discuss anything beforehand.</t>
-  </si>
-  <si>
-    <t>Hello &lt;name&gt;,  Thank you for reaching out to us and considering our IT Consulting Services. We offer a wide array of support for server installations, which includes initial assessments, planning, implementation, and ongoing maintenance. Our consultation process generally begins with an initial inquiry, followed by a detailed needs assessment and a proposal. Once both parties agree, our team will rinse and support the required solutions.  Regarding response times, we strive to acknowledge all inquiries within 24 hours and aim to swiftly address most technical concerns. For comprehensive assistance during the setup, we can provide customized documentation and suggestions tailored to your specific requirements.  Do not hesitate to let us know if you have any further inquiries or would like to arrange an initial discussion. We are keen to assist you in ensuring a smooth and effective server configuration.  Kind regards,  Customer Support Team   IT Consulting Firm   &lt;EMAILS&gt;</t>
-  </si>
-  <si>
-    <t>Consultation Process</t>
-  </si>
-  <si>
-    <t>Server Setup</t>
-  </si>
-  <si>
-    <t>Dear Customer Support Team,  I hope this message finds you well. I am writing to bring to your attention an issue regarding my recent charge for the monthly subscription of Microsoft Office 365 under the account number &lt;acc_num&gt;. I have noticed that I was overcharged on my last billing statement. I was expecting to be billed the usual amount, but it seems a higher amount was deducted. Could you please investigate and provide an immediate reimbursement for the excess charge? Your prompt attention to this matter is highly appreciated.  Thank you for your support.  Best regards,  &lt;name&gt;</t>
-  </si>
-  <si>
-    <t>Dear &lt;name&gt;,  Thank you for reaching out to us regarding your Microsoft Office 365 subscription issue. We apologize for any inconvenience caused by the overcharge on your account &lt;acc_num&gt;. We will investigate this matter promptly and work on providing a reimbursement for the excess amount charged. You can expect to hear back from us shortly with an update.  Thank you for your patience and understanding.  Best regards, Customer Support Team</t>
-  </si>
-  <si>
-    <t>Dear Pit Services Support Team,  I am writing to report that the Cisco Router ISR4331 at our enterprise is experiencing severe connectivity issues. This problem is affecting all users across our network and requires immediate technical attention. We have attempted basic troubleshooting steps such as restarting the router and checking the cables, but the issue persists. Given the critical nature of our operations, a rapid resolution is essential to minimize disruption. Please advise on the next steps, or arrange for a technician to diagnose and rectify this issue.  Thank you for your prompt assistance.  Sincerely, &lt;name&gt;</t>
-  </si>
-  <si>
-    <t>Subject: Re: Urgent Support Needed for Connectivity Issues  Dear &lt;name&gt;,  Thank you for reaching out to us regarding the connectivity issues with the Cisco Router ISR4331. We understand the urgency and impact on your operations. Please follow these steps to resolve the issue:  1. Verify that the router's firmware is up-to-date. 2. Check for any physical damage to the ports or cables. 3. Test the connection using a different router, if available.  After following these steps, if the problem persists, we will arrange for a technician to visit your site as soon as possible. Please let us know your availability for a service call.  We appreciate your patience and cooperation.  Best regards, Pit Services Support Team</t>
-  </si>
-  <si>
-    <t>It and Technical Support</t>
   </si>
   <si>
     <t>Dear Customer Support, I am writing to report a display issue we are facing with the Dell XPS 13 model 9310. The screen has been flickering intermittently, which is significantly affecting my productivity. The problem occurs unexpectedly during use, causing great inconvenience and interruption to work. Despite attempting various troubleshooting measures, including updating drivers and adjusting settings, the issue persists. Given that the laptop is less than a year old and is used extensively for professional tasks, I believe it is crucial to address this promptly to maintain its viability as a primary work device. I would appreciate guidance on how to proceed, possibly involving a warranty evaluation or repair service. Additionally, could you provide any known solutions or tips in resolving this display flicker issue? I have been a loyal customer and hope to receive prompt assistance. Please let me know if any further details are required. Thank you for your attention to this matter. Best regards, &lt;name&gt;</t>
@@ -2793,7 +2793,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2937,12 +2937,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -3288,7 +3282,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3297,9 +3291,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -14634,9 +14625,6 @@
       <c r="E302" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F302" s="1" t="s">
-        <v>708</v>
-      </c>
       <c r="G302" s="1" t="s">
         <v>47</v>
       </c>
@@ -14655,10 +14643,10 @@
     </row>
     <row r="303" spans="1:15">
       <c r="A303" s="1" t="s">
+        <v>708</v>
+      </c>
+      <c r="B303" s="1" t="s">
         <v>709</v>
-      </c>
-      <c r="B303" s="1" t="s">
-        <v>710</v>
       </c>
       <c r="C303" s="1" t="s">
         <v>41</v>
@@ -14670,7 +14658,7 @@
         <v>92</v>
       </c>
       <c r="F303" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G303" s="1" t="s">
         <v>21</v>
@@ -14690,10 +14678,10 @@
     </row>
     <row r="304" spans="1:15">
       <c r="A304" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="B304" s="1" t="s">
         <v>712</v>
-      </c>
-      <c r="B304" s="1" t="s">
-        <v>713</v>
       </c>
       <c r="C304" s="1" t="s">
         <v>36</v>
@@ -14705,7 +14693,7 @@
         <v>92</v>
       </c>
       <c r="F304" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G304" s="1" t="s">
         <v>22</v>
@@ -14717,10 +14705,10 @@
         <v>55</v>
       </c>
       <c r="J304" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="K304" s="1" t="s">
         <v>714</v>
-      </c>
-      <c r="K304" s="1" t="s">
-        <v>715</v>
       </c>
       <c r="L304" s="1" t="s">
         <v>43</v>
@@ -14737,10 +14725,10 @@
     </row>
     <row r="305" spans="1:15">
       <c r="A305" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="B305" s="1" t="s">
         <v>716</v>
-      </c>
-      <c r="B305" s="1" t="s">
-        <v>717</v>
       </c>
       <c r="C305" s="1" t="s">
         <v>17</v>
@@ -14752,7 +14740,7 @@
         <v>42</v>
       </c>
       <c r="F305" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G305" s="1" t="s">
         <v>44</v>
@@ -14775,10 +14763,10 @@
     </row>
     <row r="306" spans="1:15">
       <c r="A306" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="B306" s="1" t="s">
         <v>718</v>
-      </c>
-      <c r="B306" s="1" t="s">
-        <v>719</v>
       </c>
       <c r="C306" s="1" t="s">
         <v>36</v>
@@ -14787,10 +14775,10 @@
         <v>18</v>
       </c>
       <c r="E306" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F306" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F306" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G306" s="1" t="s">
         <v>22</v>
@@ -14831,7 +14819,7 @@
         <v>37</v>
       </c>
       <c r="F307" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G307" s="1" t="s">
         <v>21</v>
@@ -14872,10 +14860,10 @@
         <v>18</v>
       </c>
       <c r="E308" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F308" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F308" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G308" s="1" t="s">
         <v>22</v>
@@ -14919,7 +14907,7 @@
         <v>37</v>
       </c>
       <c r="F309" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G309" s="1" t="s">
         <v>21</v>
@@ -14957,7 +14945,7 @@
         <v>37</v>
       </c>
       <c r="F310" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G310" s="1" t="s">
         <v>21</v>
@@ -14992,10 +14980,10 @@
         <v>18</v>
       </c>
       <c r="E311" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F311" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G311" s="1" t="s">
         <v>21</v>
@@ -15039,7 +15027,7 @@
         <v>42</v>
       </c>
       <c r="F312" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G312" s="1" t="s">
         <v>44</v>
@@ -15074,7 +15062,7 @@
         <v>59</v>
       </c>
       <c r="F313" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G313" s="1" t="s">
         <v>47</v>
@@ -15109,7 +15097,7 @@
         <v>59</v>
       </c>
       <c r="F314" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G314" s="1" t="s">
         <v>47</v>
@@ -15144,7 +15132,7 @@
         <v>92</v>
       </c>
       <c r="F315" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G315" s="1" t="s">
         <v>21</v>
@@ -15182,7 +15170,7 @@
         <v>92</v>
       </c>
       <c r="F316" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G316" s="1" t="s">
         <v>22</v>
@@ -15217,10 +15205,10 @@
         <v>18</v>
       </c>
       <c r="E317" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F317" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F317" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G317" s="1" t="s">
         <v>21</v>
@@ -15261,7 +15249,7 @@
         <v>37</v>
       </c>
       <c r="F318" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G318" s="1" t="s">
         <v>21</v>
@@ -15296,7 +15284,7 @@
         <v>747</v>
       </c>
       <c r="F319" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G319" s="1" t="s">
         <v>55</v>
@@ -15328,10 +15316,10 @@
         <v>18</v>
       </c>
       <c r="E320" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F320" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F320" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G320" s="1" t="s">
         <v>21</v>
@@ -15369,7 +15357,7 @@
         <v>92</v>
       </c>
       <c r="F321" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G321" s="1" t="s">
         <v>21</v>
@@ -15410,10 +15398,10 @@
         <v>50</v>
       </c>
       <c r="E322" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F322" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F322" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G322" s="1" t="s">
         <v>21</v>
@@ -15454,7 +15442,7 @@
         <v>92</v>
       </c>
       <c r="F323" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G323" s="1" t="s">
         <v>21</v>
@@ -15489,10 +15477,10 @@
         <v>50</v>
       </c>
       <c r="E324" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F324" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F324" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G324" s="1" t="s">
         <v>22</v>
@@ -15533,7 +15521,7 @@
         <v>59</v>
       </c>
       <c r="F325" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G325" s="1" t="s">
         <v>21</v>
@@ -15574,7 +15562,7 @@
         <v>37</v>
       </c>
       <c r="F326" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G326" s="1" t="s">
         <v>21</v>
@@ -15615,7 +15603,7 @@
         <v>37</v>
       </c>
       <c r="F327" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G327" s="1" t="s">
         <v>47</v>
@@ -15653,7 +15641,7 @@
         <v>37</v>
       </c>
       <c r="F328" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G328" s="1" t="s">
         <v>21</v>
@@ -15694,7 +15682,7 @@
         <v>42</v>
       </c>
       <c r="F329" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G329" s="1" t="s">
         <v>44</v>
@@ -15729,7 +15717,7 @@
         <v>37</v>
       </c>
       <c r="F330" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G330" s="1" t="s">
         <v>21</v>
@@ -15770,7 +15758,7 @@
         <v>37</v>
       </c>
       <c r="F331" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G331" s="1" t="s">
         <v>21</v>
@@ -15811,10 +15799,10 @@
         <v>58</v>
       </c>
       <c r="E332" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F332" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G332" s="1" t="s">
         <v>22</v>
@@ -15849,10 +15837,10 @@
         <v>50</v>
       </c>
       <c r="E333" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F333" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F333" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G333" s="1" t="s">
         <v>23</v>
@@ -15893,7 +15881,7 @@
         <v>37</v>
       </c>
       <c r="F334" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G334" s="1" t="s">
         <v>21</v>
@@ -15928,10 +15916,10 @@
         <v>18</v>
       </c>
       <c r="E335" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F335" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F335" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G335" s="1" t="s">
         <v>21</v>
@@ -15966,10 +15954,10 @@
         <v>18</v>
       </c>
       <c r="E336" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F336" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F336" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G336" s="1" t="s">
         <v>152</v>
@@ -16013,7 +16001,7 @@
         <v>92</v>
       </c>
       <c r="F337" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G337" s="1" t="s">
         <v>21</v>
@@ -16051,10 +16039,10 @@
         <v>50</v>
       </c>
       <c r="E338" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F338" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F338" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G338" s="1" t="s">
         <v>21</v>
@@ -16089,10 +16077,10 @@
         <v>18</v>
       </c>
       <c r="E339" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F339" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F339" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G339" s="1" t="s">
         <v>23</v>
@@ -16133,7 +16121,7 @@
         <v>59</v>
       </c>
       <c r="F340" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G340" s="1" t="s">
         <v>47</v>
@@ -16174,7 +16162,7 @@
         <v>42</v>
       </c>
       <c r="F341" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G341" s="1" t="s">
         <v>44</v>
@@ -16209,7 +16197,7 @@
         <v>37</v>
       </c>
       <c r="F342" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G342" s="1" t="s">
         <v>21</v>
@@ -16241,10 +16229,10 @@
         <v>18</v>
       </c>
       <c r="E343" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F343" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F343" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G343" s="1" t="s">
         <v>21</v>
@@ -16285,7 +16273,7 @@
         <v>37</v>
       </c>
       <c r="F344" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G344" s="1" t="s">
         <v>21</v>
@@ -16332,7 +16320,7 @@
         <v>92</v>
       </c>
       <c r="F345" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G345" s="1" t="s">
         <v>22</v>
@@ -16370,7 +16358,7 @@
         <v>42</v>
       </c>
       <c r="F346" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G346" s="1" t="s">
         <v>44</v>
@@ -16405,10 +16393,10 @@
         <v>18</v>
       </c>
       <c r="E347" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F347" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F347" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G347" s="1" t="s">
         <v>22</v>
@@ -16452,7 +16440,7 @@
         <v>59</v>
       </c>
       <c r="F348" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G348" s="1" t="s">
         <v>121</v>
@@ -16487,10 +16475,10 @@
         <v>18</v>
       </c>
       <c r="E349" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F349" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F349" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G349" s="1" t="s">
         <v>21</v>
@@ -16537,7 +16525,7 @@
         <v>92</v>
       </c>
       <c r="F350" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G350" s="1" t="s">
         <v>23</v>
@@ -16575,7 +16563,7 @@
         <v>92</v>
       </c>
       <c r="F351" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G351" s="1" t="s">
         <v>22</v>
@@ -16613,10 +16601,10 @@
         <v>18</v>
       </c>
       <c r="E352" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F352" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F352" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G352" s="1" t="s">
         <v>21</v>
@@ -16657,7 +16645,7 @@
         <v>747</v>
       </c>
       <c r="F353" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G353" s="1" t="s">
         <v>60</v>
@@ -16689,10 +16677,10 @@
         <v>50</v>
       </c>
       <c r="E354" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F354" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G354" s="1" t="s">
         <v>21</v>
@@ -16733,7 +16721,7 @@
         <v>37</v>
       </c>
       <c r="F355" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G355" s="1" t="s">
         <v>21</v>
@@ -16768,10 +16756,10 @@
         <v>58</v>
       </c>
       <c r="E356" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F356" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G356" s="1" t="s">
         <v>21</v>
@@ -16812,7 +16800,7 @@
         <v>37</v>
       </c>
       <c r="F357" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G357" s="1" t="s">
         <v>21</v>
@@ -16856,7 +16844,7 @@
         <v>747</v>
       </c>
       <c r="F358" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G358" s="1" t="s">
         <v>21</v>
@@ -16897,10 +16885,10 @@
         <v>58</v>
       </c>
       <c r="E359" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F359" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G359" s="1" t="s">
         <v>124</v>
@@ -16941,7 +16929,7 @@
         <v>42</v>
       </c>
       <c r="F360" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G360" s="1" t="s">
         <v>44</v>
@@ -16979,7 +16967,7 @@
         <v>37</v>
       </c>
       <c r="F361" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G361" s="1" t="s">
         <v>21</v>
@@ -17023,7 +17011,7 @@
         <v>37</v>
       </c>
       <c r="F362" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G362" s="1" t="s">
         <v>21</v>
@@ -17067,7 +17055,7 @@
         <v>747</v>
       </c>
       <c r="F363" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G363" s="1" t="s">
         <v>22</v>
@@ -17105,10 +17093,10 @@
         <v>18</v>
       </c>
       <c r="E364" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F364" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F364" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G364" s="1" t="s">
         <v>23</v>
@@ -17149,10 +17137,10 @@
         <v>50</v>
       </c>
       <c r="E365" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F365" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F365" s="1" t="s">
-        <v>708</v>
       </c>
       <c r="G365" s="1" t="s">
         <v>21</v>
@@ -17190,7 +17178,7 @@
         <v>92</v>
       </c>
       <c r="F366" s="1" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G366" s="1" t="s">
         <v>21</v>
@@ -17231,7 +17219,7 @@
         <v>42</v>
       </c>
       <c r="F367" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G367" s="1" t="s">
         <v>44</v>
@@ -17266,7 +17254,7 @@
         <v>59</v>
       </c>
       <c r="F368" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G368" s="1" t="s">
         <v>21</v>
@@ -17307,7 +17295,7 @@
         <v>42</v>
       </c>
       <c r="F369" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G369" s="1" t="s">
         <v>44</v>
@@ -17342,7 +17330,7 @@
         <v>37</v>
       </c>
       <c r="F370" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G370" s="1" t="s">
         <v>21</v>
@@ -17377,7 +17365,7 @@
         <v>37</v>
       </c>
       <c r="F371" s="1" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="G371" s="1" t="s">
         <v>21</v>
@@ -17415,10 +17403,10 @@
         <v>18</v>
       </c>
       <c r="E372" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F372" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F372" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G372" s="1" t="s">
         <v>21</v>
@@ -17440,7 +17428,7 @@
       </c>
     </row>
     <row r="373" spans="1:15">
-      <c r="A373" s="4" t="s">
+      <c r="A373" s="3" t="s">
         <v>857</v>
       </c>
       <c r="B373" s="1" t="s">
@@ -17456,7 +17444,7 @@
         <v>37</v>
       </c>
       <c r="F373" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G373" s="1" t="s">
         <v>21</v>
@@ -17497,10 +17485,10 @@
         <v>18</v>
       </c>
       <c r="E374" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F374" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F374" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G374" s="1" t="s">
         <v>22</v>
@@ -17541,7 +17529,7 @@
         <v>37</v>
       </c>
       <c r="F375" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G375" s="1" t="s">
         <v>84</v>
@@ -17576,7 +17564,7 @@
         <v>92</v>
       </c>
       <c r="F376" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G376" s="1" t="s">
         <v>22</v>
@@ -17608,10 +17596,10 @@
         <v>58</v>
       </c>
       <c r="E377" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F377" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F377" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G377" s="1" t="s">
         <v>21</v>
@@ -17652,10 +17640,10 @@
         <v>18</v>
       </c>
       <c r="E378" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F378" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F378" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G378" s="1" t="s">
         <v>21</v>
@@ -17699,7 +17687,7 @@
         <v>37</v>
       </c>
       <c r="F379" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G379" s="1" t="s">
         <v>21</v>
@@ -17734,7 +17722,7 @@
         <v>37</v>
       </c>
       <c r="F380" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G380" s="1" t="s">
         <v>21</v>
@@ -17772,10 +17760,10 @@
         <v>18</v>
       </c>
       <c r="E381" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F381" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F381" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G381" s="1" t="s">
         <v>23</v>
@@ -17819,7 +17807,7 @@
         <v>92</v>
       </c>
       <c r="F382" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G382" s="1" t="s">
         <v>21</v>
@@ -17860,7 +17848,7 @@
         <v>37</v>
       </c>
       <c r="F383" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G383" s="1" t="s">
         <v>21</v>
@@ -17898,10 +17886,10 @@
         <v>18</v>
       </c>
       <c r="E384" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F384" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F384" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G384" s="1" t="s">
         <v>84</v>
@@ -17936,10 +17924,10 @@
         <v>18</v>
       </c>
       <c r="E385" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F385" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F385" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G385" s="1" t="s">
         <v>152</v>
@@ -17986,7 +17974,7 @@
         <v>37</v>
       </c>
       <c r="F386" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G386" s="1" t="s">
         <v>21</v>
@@ -18021,7 +18009,7 @@
         <v>747</v>
       </c>
       <c r="F387" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G387" s="1" t="s">
         <v>22</v>
@@ -18059,7 +18047,7 @@
         <v>42</v>
       </c>
       <c r="F388" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G388" s="1" t="s">
         <v>44</v>
@@ -18103,7 +18091,7 @@
         <v>92</v>
       </c>
       <c r="F389" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G389" s="1" t="s">
         <v>21</v>
@@ -18144,7 +18132,7 @@
         <v>37</v>
       </c>
       <c r="F390" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G390" s="1" t="s">
         <v>21</v>
@@ -18182,10 +18170,10 @@
         <v>50</v>
       </c>
       <c r="E391" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="F391" s="1" t="s">
         <v>720</v>
-      </c>
-      <c r="F391" s="1" t="s">
-        <v>711</v>
       </c>
       <c r="G391" s="1" t="s">
         <v>84</v>
@@ -18223,7 +18211,7 @@
         <v>92</v>
       </c>
       <c r="F392" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G392" s="1" t="s">
         <v>44</v>
@@ -18267,7 +18255,7 @@
         <v>92</v>
       </c>
       <c r="F393" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G393" s="1" t="s">
         <v>22</v>
@@ -18311,7 +18299,7 @@
         <v>42</v>
       </c>
       <c r="F394" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G394" s="1" t="s">
         <v>44</v>
@@ -18355,7 +18343,7 @@
         <v>92</v>
       </c>
       <c r="F395" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G395" s="1" t="s">
         <v>21</v>
@@ -18393,7 +18381,7 @@
         <v>37</v>
       </c>
       <c r="F396" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G396" s="1" t="s">
         <v>21</v>
@@ -18415,7 +18403,7 @@
       </c>
     </row>
     <row r="397" spans="1:15">
-      <c r="A397" s="4" t="s">
+      <c r="A397" s="3" t="s">
         <v>905</v>
       </c>
       <c r="B397" s="1" t="s">
@@ -18431,7 +18419,7 @@
         <v>92</v>
       </c>
       <c r="F397" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G397" s="1" t="s">
         <v>21</v>
@@ -18472,7 +18460,7 @@
         <v>747</v>
       </c>
       <c r="F398" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G398" s="1" t="s">
         <v>22</v>
@@ -18516,10 +18504,10 @@
         <v>50</v>
       </c>
       <c r="E399" s="1" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F399" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G399" s="1" t="s">
         <v>21</v>
@@ -18557,7 +18545,7 @@
         <v>59</v>
       </c>
       <c r="F400" s="1" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="G400" s="1" t="s">
         <v>121</v>
@@ -18595,7 +18583,7 @@
         <v>92</v>
       </c>
       <c r="F401" s="1" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G401" s="1" t="s">
         <v>60</v>

</xml_diff>